<commit_message>
Cost workbook: a play is one exercise
Recorded as decided in the offer review; the worst-case sheet already
priced Pro's credits that way.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XFCRmofgjegPCS4UYUyigf
</commit_message>
<xml_diff>
--- a/docs/business/tsuji-costs.xlsx
+++ b/docs/business/tsuji-costs.xlsx
@@ -1522,7 +1522,7 @@
     <t xml:space="preserve">Pass only; practice never spends credits.</t>
   </si>
   <si>
-    <t xml:space="preserve">To build: 1 credit per play for Pro. Assumed: a play is one exercise the model marks or writes (one sentence reviewed, one text, one paper). If a play were a whole run, Pro's worst case would be several times higher.</t>
+    <t xml:space="preserve">Decided: a play is one exercise (one sentence reviewed, one text, one paper), so one credit never buys more than one exercise's AI cost. To build: 1 credit per play for Pro.</t>
   </si>
   <si>
     <t xml:space="preserve">Mock exam</t>
@@ -2540,11 +2540,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="5244941"/>
-        <c:axId val="35062061"/>
+        <c:axId val="3403515"/>
+        <c:axId val="2935780"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="5244941"/>
+        <c:axId val="3403515"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2610,7 +2610,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="35062061"/>
+        <c:crossAx val="2935780"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2618,7 +2618,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="35062061"/>
+        <c:axId val="2935780"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2694,7 +2694,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5244941"/>
+        <c:crossAx val="3403515"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -9295,7 +9295,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="51" t="s">
         <v>485</v>
       </c>

</xml_diff>

<commit_message>
Business: practice priced per sentence, duel corrections at 1 credit
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KW983HgrX1KwassrGdK4m2
</commit_message>
<xml_diff>
--- a/docs/business/tsuji-costs.xlsx
+++ b/docs/business/tsuji-costs.xlsx
@@ -832,7 +832,7 @@
     <t xml:space="preserve">Max monthly</t>
   </si>
   <si>
-    <t xml:space="preserve">Founder prices are rounded UP to a .99 store price point, so a monthly discount can land under 25% (Pro €3.99 is −20%). In-app a founder year can lose on a learner who maxes every AI allowance; the cohort is closed (accounts created before sales open), so the loss is bounded: below.</t>
+    <t xml:space="preserve">Founder prices are rounded UP to a .99 store price point: Pro monthly €3.99 is −20% (owner's choice, 27 Oct 2026). In-app a founder year can lose on a learner who maxes every AI allowance; the cohort is closed (accounts created before sales open), so the loss is bounded: below.</t>
   </si>
   <si>
     <t xml:space="preserve">Founder rules to write: who qualifies (an account created before sales open), the month of Max (from when), the discount on the first year only, then the regular price with a reminder 30 days before renewal.</t>
@@ -874,7 +874,7 @@
     <t xml:space="preserve">Due review on Pro and Max (credits)</t>
   </si>
   <si>
-    <t xml:space="preserve">Practice exercise (average of the prices below)</t>
+    <t xml:space="preserve">Practice: average price of one unit (sentence, text, scenario) below</t>
   </si>
   <si>
     <t xml:space="preserve">Due reviews a day of a steady Pro learner (for the comparison below)</t>
@@ -991,7 +991,7 @@
     <t xml:space="preserve">A due review: 1 on Free, free on Pro.</t>
   </si>
   <si>
-    <t xml:space="preserve">Reading (one exercise)</t>
+    <t xml:space="preserve">Reading (one sentence)</t>
   </si>
   <si>
     <t xml:space="preserve">Comprehension (one text)</t>
@@ -1000,16 +1000,16 @@
     <t xml:space="preserve">From the hand-written texts; no new text is generated.</t>
   </si>
   <si>
-    <t xml:space="preserve">Dictation (one exercise)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Translation (one exercise)</t>
+    <t xml:space="preserve">Dictation (one sentence)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Translation (one sentence)</t>
   </si>
   <si>
     <t xml:space="preserve">Past the AI cap, graded by the learner.</t>
   </si>
   <si>
-    <t xml:space="preserve">Composition (one exercise)</t>
+    <t xml:space="preserve">Composition (one sentence)</t>
   </si>
   <si>
     <t xml:space="preserve">Past the AI cap, without the tutor.</t>
@@ -1036,13 +1036,13 @@
     <t xml:space="preserve">Duel with anyone else</t>
   </si>
   <si>
-    <t xml:space="preserve">Score free; details and corrections in credits (price to set).</t>
+    <t xml:space="preserve">Score free; details and corrections: 1 credit.</t>
   </si>
   <si>
     <t xml:space="preserve">Solo game</t>
   </si>
   <si>
-    <t xml:space="preserve">Price to set (end of November 2026).</t>
+    <t xml:space="preserve">Depends on the game (end of November 2026).</t>
   </si>
   <si>
     <t xml:space="preserve">AI worst case: a user who uses every AI allowance to the full, every day</t>
@@ -2146,7 +2146,7 @@
     <t xml:space="preserve">Practice modes</t>
   </si>
   <si>
-    <t xml:space="preserve">Reading 1, comprehension 2, dictation 1, translation 1, composition 1, conversation 2; free inside a mission</t>
+    <t xml:space="preserve">Per sentence: reading, dictation, translation, composition 1. Per text: comprehension 2. Per scenario: conversation 2. Free inside a mission</t>
   </si>
   <si>
     <t xml:space="preserve">Pass only; practice never spends credits.</t>
@@ -2167,7 +2167,7 @@
     <t xml:space="preserve">PvP: async duels, real time between friends, friends list</t>
   </si>
   <si>
-    <t xml:space="preserve">With a friend free, others 2 credits; score free, corrections in credits</t>
+    <t xml:space="preserve">With a friend free, others 2 credits; score free, corrections 1 credit</t>
   </si>
   <si>
     <t xml:space="preserve">Beta this week.</t>
@@ -3268,11 +3268,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="97545314"/>
-        <c:axId val="63858619"/>
+        <c:axId val="40595436"/>
+        <c:axId val="7176966"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="97545314"/>
+        <c:axId val="40595436"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3338,7 +3338,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="63858619"/>
+        <c:crossAx val="7176966"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3346,7 +3346,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="63858619"/>
+        <c:axId val="7176966"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3422,7 +3422,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97545314"/>
+        <c:crossAx val="40595436"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>

<commit_message>
Business: the early-access baseline, measured
35 learners active on two days or more in 30 replace the estimate of 25,
and the strategy points to the business plan's three paces.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KW983HgrX1KwassrGdK4m2
</commit_message>
<xml_diff>
--- a/docs/business/tsuji-costs.xlsx
+++ b/docs/business/tsuji-costs.xlsx
@@ -523,7 +523,7 @@
     <t xml:space="preserve">MAU</t>
   </si>
   <si>
-    <t xml:space="preserve">Owner, 26 Oct 2026: about 100 sign-ups, 20–30 active.</t>
+    <t xml:space="preserve">Database, 27 Oct 2026: learners active on 2 days or more in the last 30 (181 on at least one day, 21 on 3 or more). MAU here and in every sheet means that: a learner seen once is not a learner yet.</t>
   </si>
   <si>
     <t xml:space="preserve">Sales open (end of early access)</t>
@@ -3268,11 +3268,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="40595436"/>
-        <c:axId val="7176966"/>
+        <c:axId val="53878338"/>
+        <c:axId val="60884359"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="40595436"/>
+        <c:axId val="53878338"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3338,7 +3338,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="7176966"/>
+        <c:crossAx val="60884359"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3346,7 +3346,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="7176966"/>
+        <c:axId val="60884359"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3422,7 +3422,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40595436"/>
+        <c:crossAx val="53878338"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="B41" s="15" t="n">
         <f aca="false">Assumptions!$B$59</f>
-        <v>25</v>
+        <v>35</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4248,7 +4248,7 @@
       </c>
       <c r="B43" s="16" t="n">
         <f aca="false">IF(OR(B41=0,NOT(ISNUMBER(B42))),0,B42/B41)</f>
-        <v>53.32</v>
+        <v>38.0857142857143</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4266,7 +4266,7 @@
       </c>
       <c r="B45" s="18" t="n">
         <f aca="false">IF(OR(B41=0,B44=0,NOT(ISNUMBER(B42))),0,(B42/B41)^(1/B44)-1)</f>
-        <v>1.18342833104302</v>
+        <v>1.04381358016159</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4275,7 +4275,7 @@
       </c>
       <c r="B46" s="19" t="n">
         <f aca="true">IF(B45=0,0,B41*(1+B45)^(MAX(0,DATE(2026,12,31)-TODAY())/30.44))</f>
-        <v>132.470673737166</v>
+        <v>161.052800839913</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4284,7 +4284,7 @@
       </c>
       <c r="B47" s="19" t="n">
         <f aca="true">IF(B45=0,0,B41*(1+B45)^(MAX(0,Assumptions!$B$60-TODAY())/30.44))</f>
-        <v>34.8960247260582</v>
+        <v>47.4950218571389</v>
       </c>
     </row>
   </sheetData>
@@ -5698,7 +5698,7 @@
         <v>162</v>
       </c>
       <c r="B59" s="31" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="C59" s="6" t="s">
         <v>163</v>

</xml_diff>

<commit_message>
Business: Free refills 90 a day up to 120, Pro 180 up to 250
The missions now carry 35 credits a day to Free's 125-credit target, and
packs stay well above Pro (6.9 times Pro monthly).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KW983HgrX1KwassrGdK4m2
</commit_message>
<xml_diff>
--- a/docs/business/tsuji-costs.xlsx
+++ b/docs/business/tsuji-costs.xlsx
@@ -487,7 +487,7 @@
     <t xml:space="preserve">% of Pro</t>
   </si>
   <si>
-    <t xml:space="preserve">Pro learners who run past their 120 a day. Max never buys (unlimited, shop hidden).</t>
+    <t xml:space="preserve">Pro learners who run past their 180 a day. Max never buys (unlimited, shop hidden).</t>
   </si>
   <si>
     <t xml:space="preserve">Credit packs: packs bought per buyer per month</t>
@@ -973,7 +973,7 @@
     <t xml:space="preserve">Bought and earned credits never expire (owner's decision) and survive a change of plan. They never raise a plan's AI caps. The shop is hidden from Max (unlimited).</t>
   </si>
   <si>
-    <t xml:space="preserve">Proposal for the missions' 65 a day: three daily missions of 15 and a bonus of 10 for all three (55), and weekly missions worth about 70 (10 a day). A practice exercise asked by a mission costs nothing.</t>
+    <t xml:space="preserve">Proposal for the missions' 35 a day: three daily missions of 8 and a bonus of 6 for all three (30), and weekly missions worth about 35 (5 a day). A practice exercise asked by a mission costs nothing.</t>
   </si>
   <si>
     <t xml:space="preserve">What a credit buys (owner's decisions, 27 Oct 2026). Max: everything included; inside a mission: free</t>
@@ -2083,10 +2083,10 @@
     <t xml:space="preserve">Credit refill</t>
   </si>
   <si>
-    <t xml:space="preserve">60 a day; the refill stops at 90</t>
-  </si>
-  <si>
-    <t xml:space="preserve">120 a day; the refill stops at 200</t>
+    <t xml:space="preserve">90 a day; the refill stops at 120</t>
+  </si>
+  <si>
+    <t xml:space="preserve">180 a day; the refill stops at 250</t>
   </si>
   <si>
     <t xml:space="preserve">Unlimited</t>
@@ -3268,11 +3268,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="53878338"/>
-        <c:axId val="60884359"/>
+        <c:axId val="43151916"/>
+        <c:axId val="11856945"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="53878338"/>
+        <c:axId val="43151916"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3338,7 +3338,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60884359"/>
+        <c:crossAx val="11856945"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3346,7 +3346,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="60884359"/>
+        <c:axId val="11856945"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3422,7 +3422,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="53878338"/>
+        <c:crossAx val="43151916"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6841,7 +6841,7 @@
         <v>275</v>
       </c>
       <c r="B5" s="31" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6849,7 +6849,7 @@
         <v>276</v>
       </c>
       <c r="B6" s="31" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6857,7 +6857,7 @@
         <v>277</v>
       </c>
       <c r="B7" s="31" t="n">
-        <v>120</v>
+        <v>180</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6865,7 +6865,7 @@
         <v>278</v>
       </c>
       <c r="B8" s="31" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="B25" s="19" t="n">
         <f aca="false">(B7-B5)*30</f>
-        <v>1800</v>
+        <v>2700</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7138,7 +7138,7 @@
       </c>
       <c r="B27" s="19" t="n">
         <f aca="false">B25+B26</f>
-        <v>3600</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7147,7 +7147,7 @@
       </c>
       <c r="B28" s="37" t="n">
         <f aca="false">B27*MIN(D16:D19)/100</f>
-        <v>27.6646153846154</v>
+        <v>34.5807692307692</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7156,7 +7156,7 @@
       </c>
       <c r="B29" s="16" t="n">
         <f aca="false">IF(Assumptions!$B$10=0,0,B28/Assumptions!$B$10)</f>
-        <v>5.54401109912132</v>
+        <v>6.93001387390165</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7173,7 +7173,7 @@
       </c>
       <c r="B31" s="16" t="n">
         <f aca="false">IF(Assumptions!$B$10=0,0,B28/(1+B30)/Assumptions!$B$10)</f>
-        <v>3.69600739941421</v>
+        <v>4.62000924926777</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7199,7 +7199,7 @@
       </c>
       <c r="B34" s="19" t="n">
         <f aca="false">B13-B5</f>
-        <v>65</v>
+        <v>35</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Business: paid acquisition, staged and gated
A Paid acquisition sheet costs a December test, a January-March ramp and
a taper by channel (TikTok Spark Ads, Google App campaigns, Apple Ads,
micro-influencers), measured without any ad pixel or SDK; the strategy
records the phases and their gates.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KW983HgrX1KwassrGdK4m2
</commit_message>
<xml_diff>
--- a/docs/business/tsuji-costs.xlsx
+++ b/docs/business/tsuji-costs.xlsx
@@ -17,7 +17,8 @@
     <sheet name="Fixed costs" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="Unit economics" sheetId="8" state="visible" r:id="rId10"/>
     <sheet name="Projection" sheetId="9" state="visible" r:id="rId11"/>
-    <sheet name="Offer review" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="Paid acquisition" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="Offer review" sheetId="11" state="visible" r:id="rId13"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="953" uniqueCount="729">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1011" uniqueCount="784">
   <si>
     <t xml:space="preserve">Tsuji — cost overview</t>
   </si>
@@ -1924,6 +1925,171 @@
   </si>
   <si>
     <t xml:space="preserve">Steady-state snapshot: churn and growth over time are not modelled. The founder discount applies to the share of annual payers set in Assumptions; trials are costed in 'Unit economics'. Income tax is not included.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paid acquisition: buy a core of committed learners fast, then let them bring the rest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue = input · every cost per sign-up is an assumption until the December test measures it · a sign-up = a new account or guest; engaged = studies on 2 days or more in its first 30; core = still studying at day 30.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Channels (assumptions to replace with the test)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost per sign-up (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sign-up → engaged</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engaged → core</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Measured by</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TikTok Spark Ads (best organic videos boosted)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source asked at sign-up + campaign window</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No pixel, no SDK: optimised on views and link clicks.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apple Ads (search results)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apple's AdServices attribution (no ATT, no third party)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AppTweak 2025: median education CPI in the US $2.91.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google App campaigns (Android)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google Play install referrer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">53% of early-access learners are on Android.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Micro-influencers (10k–100k, FR and EN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A creator code (the referral code)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paid post marked as advertising (French law of June 2023).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Instagram Reels boost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source asked at sign-up</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Off by default: Meta education installs are dear in Europe.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Measured in early access: sign-up → engaged 17.5% (35 of 200). The test must beat it, or the money buys visitors.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What one engaged learner is worth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share of engaged learners who pay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Margin of a payer per month (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Months a payer stays</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engaged referees each engaged learner brings, over its life</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value of one engaged learner, direct (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">… with the learners it refers (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target: cost per engaged learner (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stop-loss: a channel above this multiple of the target, two weeks running, is cut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Budget by month (€): test, scale to the target, then halve once organic and referrals carry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dec 2026 (test)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jan 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feb 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mar 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apr 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">May 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What the budget buys</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sign-ups</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engaged learners</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Core learners (still studying at day 30)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost per engaged learner (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost per core learner (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value of those engaged learners, with referrals (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Net: value minus spend (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Within target?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engaged learners bought by the end of March (toward 1,333 active)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paid acquisition does not pay for itself in revenue: an engaged learner is worth about €2 with its referrals and costs about €5. It buys speed: a core that refers, reviews the app and fills the leaderboard and the library while the organic channels grow. Cut it when organic and referral sign-ups pass 60% of the total.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No advertising pixel or SDK (privacy promise, docs/adr/0012 and 0022): each channel is measured in aggregate, by its own console, Apple's AdServices or the Play install referrer, the creator's code, and a closed 'source' value asked at sign-up.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fix activation first: at 17.5% sign-up → engaged, every euro buys mostly visitors. Account after the first ride and a reliable boot come before the first euro.</t>
   </si>
   <si>
     <t xml:space="preserve">The offer as decided (26 Oct 2026), compared with the code today</t>
@@ -2585,7 +2751,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="76">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2867,6 +3033,22 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3268,11 +3450,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="43151916"/>
-        <c:axId val="11856945"/>
+        <c:axId val="59416394"/>
+        <c:axId val="55413498"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="43151916"/>
+        <c:axId val="59416394"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3338,7 +3520,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="11856945"/>
+        <c:crossAx val="55413498"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3346,7 +3528,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="11856945"/>
+        <c:axId val="55413498"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3422,7 +3604,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="43151916"/>
+        <c:crossAx val="59416394"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4303,6 +4485,824 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:I45"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="44" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="14" t="s">
+        <v>617</v>
+      </c>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+    </row>
+    <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="20" t="s">
+        <v>540</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>618</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>619</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>620</v>
+      </c>
+      <c r="E5" s="20" t="s">
+        <v>621</v>
+      </c>
+      <c r="F5" s="20" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>622</v>
+      </c>
+      <c r="B6" s="24" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D6" s="25" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>623</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>625</v>
+      </c>
+      <c r="B7" s="24" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D7" s="25" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>626</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>628</v>
+      </c>
+      <c r="B8" s="24" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D8" s="25" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>629</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>631</v>
+      </c>
+      <c r="B9" s="24" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="C9" s="23" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D9" s="25" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>632</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>634</v>
+      </c>
+      <c r="B10" s="24" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="C10" s="23" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="D10" s="25" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>635</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="44" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="14" t="s">
+        <v>638</v>
+      </c>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
+        <v>639</v>
+      </c>
+      <c r="B14" s="61" t="n">
+        <f aca="false">Assumptions!$B$15+Assumptions!$B$16</f>
+        <v>0.055</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
+        <v>640</v>
+      </c>
+      <c r="B15" s="7" t="n">
+        <f aca="false">'Unit economics'!$O$13</f>
+        <v>2.87287661877851</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>641</v>
+      </c>
+      <c r="B16" s="71" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
+        <v>642</v>
+      </c>
+      <c r="B17" s="21" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>643</v>
+      </c>
+      <c r="B18" s="37" t="n">
+        <f aca="false">B14*B15*B16</f>
+        <v>1.58008214032818</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>644</v>
+      </c>
+      <c r="B19" s="37" t="n">
+        <f aca="false">B18*(1+B17)</f>
+        <v>2.05410678242664</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
+        <v>645</v>
+      </c>
+      <c r="B20" s="24" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>646</v>
+      </c>
+      <c r="B21" s="46" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="14" t="s">
+        <v>647</v>
+      </c>
+      <c r="B23" s="14"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="14"/>
+      <c r="F23" s="14"/>
+      <c r="G23" s="14"/>
+      <c r="H23" s="14"/>
+      <c r="I23" s="14"/>
+    </row>
+    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="20" t="s">
+        <v>540</v>
+      </c>
+      <c r="B24" s="20" t="s">
+        <v>648</v>
+      </c>
+      <c r="C24" s="20" t="s">
+        <v>649</v>
+      </c>
+      <c r="D24" s="20" t="s">
+        <v>650</v>
+      </c>
+      <c r="E24" s="20" t="s">
+        <v>651</v>
+      </c>
+      <c r="F24" s="20" t="s">
+        <v>652</v>
+      </c>
+      <c r="G24" s="20" t="s">
+        <v>653</v>
+      </c>
+      <c r="H24" s="20" t="s">
+        <v>654</v>
+      </c>
+      <c r="I24" s="20" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="60" t="str">
+        <f aca="false">A6</f>
+        <v>TikTok Spark Ads (best organic videos boosted)</v>
+      </c>
+      <c r="B25" s="28" t="n">
+        <v>150</v>
+      </c>
+      <c r="C25" s="28" t="n">
+        <v>300</v>
+      </c>
+      <c r="D25" s="28" t="n">
+        <v>300</v>
+      </c>
+      <c r="E25" s="28" t="n">
+        <v>300</v>
+      </c>
+      <c r="F25" s="28" t="n">
+        <v>150</v>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>100</v>
+      </c>
+      <c r="H25" s="28" t="n">
+        <v>50</v>
+      </c>
+      <c r="I25" s="72" t="n">
+        <f aca="false">SUM(B25:H25)</f>
+        <v>1350</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="60" t="str">
+        <f aca="false">A7</f>
+        <v>Apple Ads (search results)</v>
+      </c>
+      <c r="B26" s="28" t="n">
+        <v>75</v>
+      </c>
+      <c r="C26" s="28" t="n">
+        <v>100</v>
+      </c>
+      <c r="D26" s="28" t="n">
+        <v>100</v>
+      </c>
+      <c r="E26" s="28" t="n">
+        <v>100</v>
+      </c>
+      <c r="F26" s="28" t="n">
+        <v>75</v>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>50</v>
+      </c>
+      <c r="H26" s="28" t="n">
+        <v>50</v>
+      </c>
+      <c r="I26" s="72" t="n">
+        <f aca="false">SUM(B26:H26)</f>
+        <v>550</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="60" t="str">
+        <f aca="false">A8</f>
+        <v>Google App campaigns (Android)</v>
+      </c>
+      <c r="B27" s="28" t="n">
+        <v>75</v>
+      </c>
+      <c r="C27" s="28" t="n">
+        <v>150</v>
+      </c>
+      <c r="D27" s="28" t="n">
+        <v>150</v>
+      </c>
+      <c r="E27" s="28" t="n">
+        <v>150</v>
+      </c>
+      <c r="F27" s="28" t="n">
+        <v>75</v>
+      </c>
+      <c r="G27" s="28" t="n">
+        <v>50</v>
+      </c>
+      <c r="H27" s="28" t="n">
+        <v>25</v>
+      </c>
+      <c r="I27" s="72" t="n">
+        <f aca="false">SUM(B27:H27)</f>
+        <v>675</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="60" t="str">
+        <f aca="false">A9</f>
+        <v>Micro-influencers (10k–100k, FR and EN)</v>
+      </c>
+      <c r="B28" s="28" t="n">
+        <v>100</v>
+      </c>
+      <c r="C28" s="28" t="n">
+        <v>150</v>
+      </c>
+      <c r="D28" s="28" t="n">
+        <v>150</v>
+      </c>
+      <c r="E28" s="28" t="n">
+        <v>150</v>
+      </c>
+      <c r="F28" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="72" t="n">
+        <f aca="false">SUM(B28:H28)</f>
+        <v>550</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="60" t="str">
+        <f aca="false">A10</f>
+        <v>Instagram Reels boost</v>
+      </c>
+      <c r="B29" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="72" t="n">
+        <f aca="false">SUM(B29:H29)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="8" t="s">
+        <v>656</v>
+      </c>
+      <c r="B30" s="73" t="n">
+        <f aca="false">SUM(B25:B29)</f>
+        <v>400</v>
+      </c>
+      <c r="C30" s="73" t="n">
+        <f aca="false">SUM(C25:C29)</f>
+        <v>700</v>
+      </c>
+      <c r="D30" s="73" t="n">
+        <f aca="false">SUM(D25:D29)</f>
+        <v>700</v>
+      </c>
+      <c r="E30" s="73" t="n">
+        <f aca="false">SUM(E25:E29)</f>
+        <v>700</v>
+      </c>
+      <c r="F30" s="73" t="n">
+        <f aca="false">SUM(F25:F29)</f>
+        <v>300</v>
+      </c>
+      <c r="G30" s="73" t="n">
+        <f aca="false">SUM(G25:G29)</f>
+        <v>200</v>
+      </c>
+      <c r="H30" s="73" t="n">
+        <f aca="false">SUM(H25:H29)</f>
+        <v>125</v>
+      </c>
+      <c r="I30" s="73" t="n">
+        <f aca="false">SUM(I25:I29)</f>
+        <v>3125</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="14" t="s">
+        <v>657</v>
+      </c>
+      <c r="B32" s="14"/>
+      <c r="C32" s="14"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="14"/>
+      <c r="F32" s="14"/>
+      <c r="G32" s="14"/>
+      <c r="H32" s="14"/>
+      <c r="I32" s="14"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="6" t="s">
+        <v>658</v>
+      </c>
+      <c r="B33" s="19" t="n">
+        <f aca="false">SUMPRODUCT(B25:B29/$B$6:$B$10)</f>
+        <v>297.5</v>
+      </c>
+      <c r="C33" s="19" t="n">
+        <f aca="false">SUMPRODUCT(C25:C29/$B$6:$B$10)</f>
+        <v>535</v>
+      </c>
+      <c r="D33" s="19" t="n">
+        <f aca="false">SUMPRODUCT(D25:D29/$B$6:$B$10)</f>
+        <v>535</v>
+      </c>
+      <c r="E33" s="19" t="n">
+        <f aca="false">SUMPRODUCT(E25:E29/$B$6:$B$10)</f>
+        <v>535</v>
+      </c>
+      <c r="F33" s="19" t="n">
+        <f aca="false">SUMPRODUCT(F25:F29/$B$6:$B$10)</f>
+        <v>217.5</v>
+      </c>
+      <c r="G33" s="19" t="n">
+        <f aca="false">SUMPRODUCT(G25:G29/$B$6:$B$10)</f>
+        <v>145</v>
+      </c>
+      <c r="H33" s="19" t="n">
+        <f aca="false">SUMPRODUCT(H25:H29/$B$6:$B$10)</f>
+        <v>82.5</v>
+      </c>
+      <c r="I33" s="69" t="n">
+        <f aca="false">SUM(B33:H33)</f>
+        <v>2347.5</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="6" t="s">
+        <v>659</v>
+      </c>
+      <c r="B34" s="19" t="n">
+        <f aca="false">SUMPRODUCT(B25:B29/$B$6:$B$10*$C$6:$C$10)</f>
+        <v>70.5</v>
+      </c>
+      <c r="C34" s="19" t="n">
+        <f aca="false">SUMPRODUCT(C25:C29/$B$6:$B$10*$C$6:$C$10)</f>
+        <v>123</v>
+      </c>
+      <c r="D34" s="19" t="n">
+        <f aca="false">SUMPRODUCT(D25:D29/$B$6:$B$10*$C$6:$C$10)</f>
+        <v>123</v>
+      </c>
+      <c r="E34" s="19" t="n">
+        <f aca="false">SUMPRODUCT(E25:E29/$B$6:$B$10*$C$6:$C$10)</f>
+        <v>123</v>
+      </c>
+      <c r="F34" s="19" t="n">
+        <f aca="false">SUMPRODUCT(F25:F29/$B$6:$B$10*$C$6:$C$10)</f>
+        <v>46.5</v>
+      </c>
+      <c r="G34" s="19" t="n">
+        <f aca="false">SUMPRODUCT(G25:G29/$B$6:$B$10*$C$6:$C$10)</f>
+        <v>31</v>
+      </c>
+      <c r="H34" s="19" t="n">
+        <f aca="false">SUMPRODUCT(H25:H29/$B$6:$B$10*$C$6:$C$10)</f>
+        <v>18.5</v>
+      </c>
+      <c r="I34" s="69" t="n">
+        <f aca="false">SUM(B34:H34)</f>
+        <v>535.5</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="8" t="s">
+        <v>660</v>
+      </c>
+      <c r="B35" s="69" t="n">
+        <f aca="false">SUMPRODUCT(B25:B29/$B$6:$B$10*$C$6:$C$10*$D$6:$D$10)</f>
+        <v>29.85</v>
+      </c>
+      <c r="C35" s="69" t="n">
+        <f aca="false">SUMPRODUCT(C25:C29/$B$6:$B$10*$C$6:$C$10*$D$6:$D$10)</f>
+        <v>51.6</v>
+      </c>
+      <c r="D35" s="69" t="n">
+        <f aca="false">SUMPRODUCT(D25:D29/$B$6:$B$10*$C$6:$C$10*$D$6:$D$10)</f>
+        <v>51.6</v>
+      </c>
+      <c r="E35" s="69" t="n">
+        <f aca="false">SUMPRODUCT(E25:E29/$B$6:$B$10*$C$6:$C$10*$D$6:$D$10)</f>
+        <v>51.6</v>
+      </c>
+      <c r="F35" s="69" t="n">
+        <f aca="false">SUMPRODUCT(F25:F29/$B$6:$B$10*$C$6:$C$10*$D$6:$D$10)</f>
+        <v>19.05</v>
+      </c>
+      <c r="G35" s="69" t="n">
+        <f aca="false">SUMPRODUCT(G25:G29/$B$6:$B$10*$C$6:$C$10*$D$6:$D$10)</f>
+        <v>12.7</v>
+      </c>
+      <c r="H35" s="69" t="n">
+        <f aca="false">SUMPRODUCT(H25:H29/$B$6:$B$10*$C$6:$C$10*$D$6:$D$10)</f>
+        <v>7.7</v>
+      </c>
+      <c r="I35" s="69" t="n">
+        <f aca="false">SUM(B35:H35)</f>
+        <v>224.1</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="6" t="s">
+        <v>661</v>
+      </c>
+      <c r="B36" s="37" t="n">
+        <f aca="false">IF(B34=0,0,B30/B34)</f>
+        <v>5.67375886524823</v>
+      </c>
+      <c r="C36" s="37" t="n">
+        <f aca="false">IF(C34=0,0,C30/C34)</f>
+        <v>5.69105691056911</v>
+      </c>
+      <c r="D36" s="37" t="n">
+        <f aca="false">IF(D34=0,0,D30/D34)</f>
+        <v>5.69105691056911</v>
+      </c>
+      <c r="E36" s="37" t="n">
+        <f aca="false">IF(E34=0,0,E30/E34)</f>
+        <v>5.69105691056911</v>
+      </c>
+      <c r="F36" s="37" t="n">
+        <f aca="false">IF(F34=0,0,F30/F34)</f>
+        <v>6.45161290322581</v>
+      </c>
+      <c r="G36" s="37" t="n">
+        <f aca="false">IF(G34=0,0,G30/G34)</f>
+        <v>6.45161290322581</v>
+      </c>
+      <c r="H36" s="37" t="n">
+        <f aca="false">IF(H34=0,0,H30/H34)</f>
+        <v>6.75675675675676</v>
+      </c>
+      <c r="I36" s="37" t="n">
+        <f aca="false">IF(I34=0,0,I30/I34)</f>
+        <v>5.83566760037348</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="s">
+        <v>662</v>
+      </c>
+      <c r="B37" s="37" t="n">
+        <f aca="false">IF(B35=0,0,B30/B35)</f>
+        <v>13.4003350083752</v>
+      </c>
+      <c r="C37" s="37" t="n">
+        <f aca="false">IF(C35=0,0,C30/C35)</f>
+        <v>13.5658914728682</v>
+      </c>
+      <c r="D37" s="37" t="n">
+        <f aca="false">IF(D35=0,0,D30/D35)</f>
+        <v>13.5658914728682</v>
+      </c>
+      <c r="E37" s="37" t="n">
+        <f aca="false">IF(E35=0,0,E30/E35)</f>
+        <v>13.5658914728682</v>
+      </c>
+      <c r="F37" s="37" t="n">
+        <f aca="false">IF(F35=0,0,F30/F35)</f>
+        <v>15.748031496063</v>
+      </c>
+      <c r="G37" s="37" t="n">
+        <f aca="false">IF(G35=0,0,G30/G35)</f>
+        <v>15.748031496063</v>
+      </c>
+      <c r="H37" s="37" t="n">
+        <f aca="false">IF(H35=0,0,H30/H35)</f>
+        <v>16.2337662337662</v>
+      </c>
+      <c r="I37" s="37" t="n">
+        <f aca="false">IF(I35=0,0,I30/I35)</f>
+        <v>13.9446675591254</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6" t="s">
+        <v>663</v>
+      </c>
+      <c r="B38" s="74" t="n">
+        <f aca="false">B34*$B$19</f>
+        <v>144.814528161078</v>
+      </c>
+      <c r="C38" s="74" t="n">
+        <f aca="false">C34*$B$19</f>
+        <v>252.655134238476</v>
+      </c>
+      <c r="D38" s="74" t="n">
+        <f aca="false">D34*$B$19</f>
+        <v>252.655134238476</v>
+      </c>
+      <c r="E38" s="74" t="n">
+        <f aca="false">E34*$B$19</f>
+        <v>252.655134238476</v>
+      </c>
+      <c r="F38" s="74" t="n">
+        <f aca="false">F34*$B$19</f>
+        <v>95.5159653828386</v>
+      </c>
+      <c r="G38" s="74" t="n">
+        <f aca="false">G34*$B$19</f>
+        <v>63.6773102552258</v>
+      </c>
+      <c r="H38" s="74" t="n">
+        <f aca="false">H34*$B$19</f>
+        <v>38.0009754748928</v>
+      </c>
+      <c r="I38" s="72" t="n">
+        <f aca="false">SUM(B38:H38)</f>
+        <v>1099.97418198946</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="8" t="s">
+        <v>664</v>
+      </c>
+      <c r="B39" s="72" t="n">
+        <f aca="false">B38-B30</f>
+        <v>-255.185471838922</v>
+      </c>
+      <c r="C39" s="72" t="n">
+        <f aca="false">C38-C30</f>
+        <v>-447.344865761524</v>
+      </c>
+      <c r="D39" s="72" t="n">
+        <f aca="false">D38-D30</f>
+        <v>-447.344865761524</v>
+      </c>
+      <c r="E39" s="72" t="n">
+        <f aca="false">E38-E30</f>
+        <v>-447.344865761524</v>
+      </c>
+      <c r="F39" s="72" t="n">
+        <f aca="false">F38-F30</f>
+        <v>-204.484034617161</v>
+      </c>
+      <c r="G39" s="72" t="n">
+        <f aca="false">G38-G30</f>
+        <v>-136.322689744774</v>
+      </c>
+      <c r="H39" s="72" t="n">
+        <f aca="false">H38-H30</f>
+        <v>-86.9990245251072</v>
+      </c>
+      <c r="I39" s="72" t="n">
+        <f aca="false">SUM(B39:H39)</f>
+        <v>-2025.02581801054</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="8" t="s">
+        <v>665</v>
+      </c>
+      <c r="I40" s="8" t="str">
+        <f aca="false">IF(I36&lt;=$B$20,"yes","NO: fix activation before spending more")</f>
+        <v>NO: fix activation before spending more</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="8" t="s">
+        <v>666</v>
+      </c>
+      <c r="I41" s="69" t="n">
+        <f aca="false">SUM(B34:E34)</f>
+        <v>439.5</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="40" t="s">
+        <v>667</v>
+      </c>
+      <c r="B43" s="40"/>
+      <c r="C43" s="40"/>
+      <c r="D43" s="40"/>
+      <c r="E43" s="40"/>
+      <c r="F43" s="40"/>
+      <c r="G43" s="40"/>
+      <c r="H43" s="40"/>
+      <c r="I43" s="40"/>
+    </row>
+    <row r="44" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="40" t="s">
+        <v>668</v>
+      </c>
+      <c r="B44" s="40"/>
+      <c r="C44" s="40"/>
+      <c r="D44" s="40"/>
+      <c r="E44" s="40"/>
+      <c r="F44" s="40"/>
+      <c r="G44" s="40"/>
+      <c r="H44" s="40"/>
+      <c r="I44" s="40"/>
+    </row>
+    <row r="45" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="40" t="s">
+        <v>669</v>
+      </c>
+      <c r="B45" s="40"/>
+      <c r="C45" s="40"/>
+      <c r="D45" s="40"/>
+      <c r="E45" s="40"/>
+      <c r="F45" s="40"/>
+      <c r="G45" s="40"/>
+      <c r="H45" s="40"/>
+      <c r="I45" s="40"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A43:I43"/>
+    <mergeCell ref="A44:I44"/>
+    <mergeCell ref="A45:I45"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:F40"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -4316,7 +5316,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>615</v>
+        <v>670</v>
       </c>
       <c r="B1" s="70"/>
       <c r="C1" s="70"/>
@@ -4326,7 +5326,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="44" t="s">
-        <v>616</v>
+        <v>671</v>
       </c>
       <c r="B2" s="70"/>
       <c r="C2" s="70"/>
@@ -4344,10 +5344,10 @@
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="20" t="s">
-        <v>617</v>
+        <v>672</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>618</v>
+        <v>673</v>
       </c>
       <c r="C4" s="20" t="s">
         <v>188</v>
@@ -4356,175 +5356,175 @@
         <v>191</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>619</v>
+        <v>674</v>
       </c>
       <c r="F4" s="20" t="s">
-        <v>620</v>
+        <v>675</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="71" t="s">
-        <v>621</v>
+      <c r="A5" s="75" t="s">
+        <v>676</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>622</v>
+        <v>677</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>623</v>
+        <v>678</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>624</v>
+        <v>679</v>
       </c>
       <c r="E5" s="22" t="s">
-        <v>625</v>
+        <v>680</v>
       </c>
       <c r="F5" s="22" t="s">
-        <v>626</v>
+        <v>681</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="71" t="s">
-        <v>627</v>
+      <c r="A6" s="75" t="s">
+        <v>682</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>628</v>
+        <v>683</v>
       </c>
       <c r="C6" s="22" t="s">
-        <v>629</v>
+        <v>684</v>
       </c>
       <c r="D6" s="22" t="s">
-        <v>630</v>
+        <v>685</v>
       </c>
       <c r="E6" s="22" t="s">
-        <v>631</v>
+        <v>686</v>
       </c>
       <c r="F6" s="22" t="s">
-        <v>632</v>
+        <v>687</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="71" t="s">
-        <v>633</v>
+      <c r="A7" s="75" t="s">
+        <v>688</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>634</v>
+        <v>689</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>635</v>
+        <v>690</v>
       </c>
       <c r="D7" s="22" t="s">
-        <v>636</v>
+        <v>691</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>637</v>
+        <v>692</v>
       </c>
       <c r="F7" s="22" t="s">
-        <v>638</v>
+        <v>693</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="71" t="s">
-        <v>639</v>
+      <c r="A8" s="75" t="s">
+        <v>694</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>640</v>
+        <v>695</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>641</v>
+        <v>696</v>
       </c>
       <c r="D8" s="22" t="s">
         <v>209</v>
       </c>
       <c r="E8" s="22" t="s">
-        <v>642</v>
+        <v>697</v>
       </c>
       <c r="F8" s="22" t="s">
-        <v>643</v>
+        <v>698</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="71" t="s">
-        <v>644</v>
+      <c r="A9" s="75" t="s">
+        <v>699</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>645</v>
+        <v>700</v>
       </c>
       <c r="C9" s="22" t="s">
-        <v>618</v>
+        <v>673</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>618</v>
+        <v>673</v>
       </c>
       <c r="E9" s="22" t="s">
-        <v>646</v>
+        <v>701</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>643</v>
+        <v>698</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="71" t="s">
-        <v>647</v>
+      <c r="A10" s="75" t="s">
+        <v>702</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>648</v>
+        <v>703</v>
       </c>
       <c r="C10" s="22" t="s">
-        <v>641</v>
+        <v>696</v>
       </c>
       <c r="D10" s="22" t="s">
-        <v>649</v>
+        <v>704</v>
       </c>
       <c r="E10" s="22" t="s">
-        <v>650</v>
+        <v>705</v>
       </c>
       <c r="F10" s="22" t="s">
-        <v>643</v>
+        <v>698</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="71" t="s">
-        <v>651</v>
+      <c r="A11" s="75" t="s">
+        <v>706</v>
       </c>
       <c r="B11" s="22" t="s">
-        <v>645</v>
+        <v>700</v>
       </c>
       <c r="C11" s="22" t="s">
-        <v>645</v>
+        <v>700</v>
       </c>
       <c r="D11" s="22" t="s">
-        <v>649</v>
+        <v>704</v>
       </c>
       <c r="E11" s="22" t="s">
-        <v>652</v>
+        <v>707</v>
       </c>
       <c r="F11" s="22" t="s">
-        <v>653</v>
+        <v>708</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="71" t="s">
-        <v>654</v>
+      <c r="A12" s="75" t="s">
+        <v>709</v>
       </c>
       <c r="B12" s="22" t="s">
-        <v>655</v>
+        <v>710</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>641</v>
+        <v>696</v>
       </c>
       <c r="D12" s="22" t="s">
-        <v>649</v>
+        <v>704</v>
       </c>
       <c r="E12" s="22" t="s">
-        <v>656</v>
+        <v>711</v>
       </c>
       <c r="F12" s="22" t="s">
-        <v>657</v>
+        <v>712</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="71" t="s">
-        <v>658</v>
+      <c r="A13" s="75" t="s">
+        <v>713</v>
       </c>
       <c r="B13" s="22" t="s">
         <v>286</v>
@@ -4533,313 +5533,313 @@
         <v>286</v>
       </c>
       <c r="D13" s="22" t="s">
-        <v>649</v>
+        <v>704</v>
       </c>
       <c r="E13" s="22" t="s">
-        <v>659</v>
+        <v>714</v>
       </c>
       <c r="F13" s="22" t="s">
-        <v>660</v>
+        <v>715</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="71" t="s">
-        <v>661</v>
+      <c r="A14" s="75" t="s">
+        <v>716</v>
       </c>
       <c r="B14" s="22" t="s">
-        <v>662</v>
+        <v>717</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>641</v>
+        <v>696</v>
       </c>
       <c r="D14" s="22" t="s">
-        <v>649</v>
+        <v>704</v>
       </c>
       <c r="E14" s="22" t="s">
-        <v>663</v>
+        <v>718</v>
       </c>
       <c r="F14" s="22" t="s">
-        <v>664</v>
+        <v>719</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="71" t="s">
-        <v>665</v>
+      <c r="A15" s="75" t="s">
+        <v>720</v>
       </c>
       <c r="B15" s="22" t="s">
-        <v>666</v>
+        <v>721</v>
       </c>
       <c r="C15" s="22" t="s">
-        <v>666</v>
+        <v>721</v>
       </c>
       <c r="D15" s="22" t="s">
-        <v>667</v>
+        <v>722</v>
       </c>
       <c r="E15" s="22" t="s">
-        <v>668</v>
+        <v>723</v>
       </c>
       <c r="F15" s="22" t="s">
-        <v>669</v>
+        <v>724</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="71" t="s">
-        <v>670</v>
+      <c r="A16" s="75" t="s">
+        <v>725</v>
       </c>
       <c r="B16" s="22" t="s">
-        <v>671</v>
+        <v>726</v>
       </c>
       <c r="C16" s="22" t="s">
-        <v>641</v>
+        <v>696</v>
       </c>
       <c r="D16" s="22" t="s">
-        <v>672</v>
+        <v>727</v>
       </c>
       <c r="E16" s="22" t="s">
-        <v>659</v>
+        <v>714</v>
       </c>
       <c r="F16" s="22" t="s">
-        <v>673</v>
+        <v>728</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="71" t="s">
-        <v>674</v>
+      <c r="A17" s="75" t="s">
+        <v>729</v>
       </c>
       <c r="B17" s="22" t="s">
-        <v>675</v>
+        <v>730</v>
       </c>
       <c r="C17" s="22" t="s">
-        <v>641</v>
+        <v>696</v>
       </c>
       <c r="D17" s="22" t="s">
-        <v>672</v>
+        <v>727</v>
       </c>
       <c r="E17" s="22" t="s">
-        <v>659</v>
+        <v>714</v>
       </c>
       <c r="F17" s="22" t="s">
-        <v>676</v>
+        <v>731</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="71" t="s">
-        <v>677</v>
+      <c r="A18" s="75" t="s">
+        <v>732</v>
       </c>
       <c r="B18" s="22" t="s">
-        <v>678</v>
+        <v>733</v>
       </c>
       <c r="C18" s="22" t="s">
-        <v>679</v>
+        <v>734</v>
       </c>
       <c r="D18" s="22" t="s">
-        <v>680</v>
+        <v>735</v>
       </c>
       <c r="E18" s="22" t="s">
-        <v>681</v>
+        <v>736</v>
       </c>
       <c r="F18" s="22" t="s">
-        <v>682</v>
+        <v>737</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="71" t="s">
-        <v>683</v>
+      <c r="A19" s="75" t="s">
+        <v>738</v>
       </c>
       <c r="B19" s="22" t="s">
-        <v>684</v>
+        <v>739</v>
       </c>
       <c r="C19" s="22" t="s">
-        <v>641</v>
+        <v>696</v>
       </c>
       <c r="D19" s="22" t="s">
-        <v>649</v>
+        <v>704</v>
       </c>
       <c r="E19" s="22" t="s">
-        <v>685</v>
+        <v>740</v>
       </c>
       <c r="F19" s="22" t="s">
-        <v>686</v>
+        <v>741</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="71" t="s">
-        <v>687</v>
+      <c r="A20" s="75" t="s">
+        <v>742</v>
       </c>
       <c r="B20" s="22" t="s">
-        <v>688</v>
+        <v>743</v>
       </c>
       <c r="C20" s="22" t="s">
-        <v>689</v>
+        <v>744</v>
       </c>
       <c r="D20" s="22" t="s">
-        <v>690</v>
+        <v>745</v>
       </c>
       <c r="E20" s="22" t="s">
-        <v>691</v>
+        <v>746</v>
       </c>
       <c r="F20" s="22" t="s">
-        <v>692</v>
+        <v>747</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="71" t="s">
-        <v>693</v>
+      <c r="A21" s="75" t="s">
+        <v>748</v>
       </c>
       <c r="B21" s="22" t="s">
-        <v>694</v>
+        <v>749</v>
       </c>
       <c r="C21" s="22" t="s">
-        <v>695</v>
+        <v>750</v>
       </c>
       <c r="D21" s="22" t="s">
-        <v>696</v>
+        <v>751</v>
       </c>
       <c r="E21" s="22" t="s">
-        <v>697</v>
+        <v>752</v>
       </c>
       <c r="F21" s="22" t="s">
-        <v>698</v>
+        <v>753</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="71" t="s">
-        <v>699</v>
+      <c r="A22" s="75" t="s">
+        <v>754</v>
       </c>
       <c r="B22" s="22" t="s">
-        <v>700</v>
+        <v>755</v>
       </c>
       <c r="C22" s="22" t="s">
-        <v>700</v>
+        <v>755</v>
       </c>
       <c r="D22" s="22" t="s">
-        <v>701</v>
+        <v>756</v>
       </c>
       <c r="E22" s="22" t="s">
-        <v>659</v>
+        <v>714</v>
       </c>
       <c r="F22" s="22" t="s">
-        <v>702</v>
+        <v>757</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="71" t="s">
-        <v>703</v>
+      <c r="A23" s="75" t="s">
+        <v>758</v>
       </c>
       <c r="B23" s="22" t="s">
         <v>209</v>
       </c>
       <c r="C23" s="22" t="s">
-        <v>704</v>
+        <v>759</v>
       </c>
       <c r="D23" s="22" t="s">
-        <v>704</v>
+        <v>759</v>
       </c>
       <c r="E23" s="22" t="s">
         <v>209</v>
       </c>
       <c r="F23" s="22" t="s">
-        <v>643</v>
+        <v>698</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="71" t="s">
-        <v>705</v>
+      <c r="A24" s="75" t="s">
+        <v>760</v>
       </c>
       <c r="B24" s="22" t="s">
         <v>209</v>
       </c>
       <c r="C24" s="22" t="s">
-        <v>706</v>
+        <v>761</v>
       </c>
       <c r="D24" s="22" t="s">
-        <v>706</v>
+        <v>761</v>
       </c>
       <c r="E24" s="22" t="s">
         <v>209</v>
       </c>
       <c r="F24" s="22" t="s">
-        <v>707</v>
+        <v>762</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="71" t="s">
-        <v>708</v>
+      <c r="A25" s="75" t="s">
+        <v>763</v>
       </c>
       <c r="B25" s="22" t="s">
         <v>209</v>
       </c>
       <c r="C25" s="22" t="s">
-        <v>709</v>
+        <v>764</v>
       </c>
       <c r="D25" s="22" t="s">
-        <v>709</v>
+        <v>764</v>
       </c>
       <c r="E25" s="22" t="s">
-        <v>659</v>
+        <v>714</v>
       </c>
       <c r="F25" s="22" t="s">
-        <v>710</v>
+        <v>765</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="71" t="s">
-        <v>711</v>
+      <c r="A26" s="75" t="s">
+        <v>766</v>
       </c>
       <c r="B26" s="22" t="s">
         <v>209</v>
       </c>
       <c r="C26" s="22" t="s">
-        <v>712</v>
+        <v>767</v>
       </c>
       <c r="D26" s="22" t="s">
-        <v>713</v>
+        <v>768</v>
       </c>
       <c r="E26" s="22" t="s">
-        <v>659</v>
+        <v>714</v>
       </c>
       <c r="F26" s="22" t="s">
-        <v>714</v>
+        <v>769</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="71" t="s">
-        <v>715</v>
+      <c r="A27" s="75" t="s">
+        <v>770</v>
       </c>
       <c r="B27" s="22" t="s">
         <v>209</v>
       </c>
       <c r="C27" s="22" t="s">
-        <v>716</v>
+        <v>771</v>
       </c>
       <c r="D27" s="22" t="s">
-        <v>717</v>
+        <v>772</v>
       </c>
       <c r="E27" s="22" t="s">
-        <v>718</v>
+        <v>773</v>
       </c>
       <c r="F27" s="22" t="s">
-        <v>643</v>
+        <v>698</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="71" t="s">
-        <v>719</v>
+      <c r="A28" s="75" t="s">
+        <v>774</v>
       </c>
       <c r="B28" s="22" t="s">
         <v>209</v>
       </c>
       <c r="C28" s="22" t="s">
-        <v>720</v>
+        <v>775</v>
       </c>
       <c r="D28" s="22" t="s">
-        <v>720</v>
+        <v>775</v>
       </c>
       <c r="E28" s="22" t="s">
-        <v>659</v>
+        <v>714</v>
       </c>
       <c r="F28" s="22" t="s">
-        <v>643</v>
+        <v>698</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4852,7 +5852,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="14" t="s">
-        <v>721</v>
+        <v>776</v>
       </c>
       <c r="B30" s="14"/>
       <c r="C30" s="14"/>
@@ -4865,7 +5865,7 @@
         <v>1</v>
       </c>
       <c r="B31" s="40" t="s">
-        <v>722</v>
+        <v>777</v>
       </c>
       <c r="C31" s="40"/>
       <c r="D31" s="40"/>
@@ -4877,7 +5877,7 @@
         <v>2</v>
       </c>
       <c r="B32" s="40" t="s">
-        <v>723</v>
+        <v>778</v>
       </c>
       <c r="C32" s="40"/>
       <c r="D32" s="40"/>
@@ -4889,7 +5889,7 @@
         <v>3</v>
       </c>
       <c r="B33" s="40" t="s">
-        <v>724</v>
+        <v>779</v>
       </c>
       <c r="C33" s="40"/>
       <c r="D33" s="40"/>
@@ -4901,7 +5901,7 @@
         <v>4</v>
       </c>
       <c r="B34" s="40" t="s">
-        <v>725</v>
+        <v>780</v>
       </c>
       <c r="C34" s="40"/>
       <c r="D34" s="40"/>
@@ -4913,7 +5913,7 @@
         <v>5</v>
       </c>
       <c r="B35" s="40" t="s">
-        <v>726</v>
+        <v>781</v>
       </c>
       <c r="C35" s="40"/>
       <c r="D35" s="40"/>
@@ -4925,7 +5925,7 @@
         <v>6</v>
       </c>
       <c r="B36" s="40" t="s">
-        <v>727</v>
+        <v>782</v>
       </c>
       <c r="C36" s="40"/>
       <c r="D36" s="40"/>
@@ -4937,7 +5937,7 @@
         <v>7</v>
       </c>
       <c r="B37" s="40" t="s">
-        <v>728</v>
+        <v>783</v>
       </c>
       <c r="C37" s="40"/>
       <c r="D37" s="40"/>

</xml_diff>